<commit_message>
Use SAP delivery notes for parts usage
</commit_message>
<xml_diff>
--- a/Reference/SPL Planning Data Fields edited.xlsx
+++ b/Reference/SPL Planning Data Fields edited.xlsx
@@ -7931,7 +7931,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8056,7 +8056,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8250,7 +8250,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8372,7 +8372,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8437,7 +8437,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8571,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8641,7 +8641,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>
@@ -8705,7 +8705,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>Usage is allowed from the manually generated SAP Stock Audit Report; work-order linkage may need SAP verification.</t>
+          <t>Delivery Notes are the source of truth for actual part usage; call/customer/serial values are enriched from ODLN.NumAtCard and ODLN.Comments when present.</t>
         </is>
       </c>
     </row>

</xml_diff>